<commit_message>
updated co2 storage limits for phase 1 capacities
</commit_message>
<xml_diff>
--- a/mes_north_sea/clean_data/nodes/nodes_2040.xlsx
+++ b/mes_north_sea/clean_data/nodes/nodes_2040.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maiant/PycharmProjects/Key-Infrastructure-North-Sea-CodeAndData/mes_north_sea/clean_data/nodes/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/8051917/PycharmProjects/AdOpT-NET0_DAC-Offshore/mes_north_sea/clean_data/nodes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F570C56-6D06-1A44-BEF2-F34F45A49353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C5E79E8-DE2C-D64F-AF92-260D72C1D8BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="660" windowWidth="19260" windowHeight="15660" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="15120" windowHeight="17480" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes_used" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="225">
   <si>
     <t>Node</t>
   </si>
@@ -682,9 +682,6 @@
     <t>Havstjerne &amp; Poseidon</t>
   </si>
   <si>
-    <t>Albondigas &amp; Kinno &amp; Iroko</t>
-  </si>
-  <si>
     <t>Polaris &amp; Snohvit</t>
   </si>
   <si>
@@ -731,6 +728,15 @@
   </si>
   <si>
     <t>No capacity announced for Net Zero Humber, placeholder at 500,000,000 like Greensand in NO with the same injection rate</t>
+  </si>
+  <si>
+    <t>phase 1</t>
+  </si>
+  <si>
+    <t>Column1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Albondigas &amp; Kinno </t>
   </si>
 </sst>
 </file>
@@ -902,7 +908,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
@@ -991,6 +997,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1073,9 +1080,15 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8198ECEC-84CC-8C4C-89D8-C0C7326FC773}" name="Table2" displayName="Table2" ref="A1:G16" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="A1:G16" xr:uid="{8198ECEC-84CC-8C4C-89D8-C0C7326FC773}"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8198ECEC-84CC-8C4C-89D8-C0C7326FC773}" name="Table2" displayName="Table2" ref="A1:H16" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:H16" xr:uid="{8198ECEC-84CC-8C4C-89D8-C0C7326FC773}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="DK"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{D2330856-3D51-2447-BAD1-42FD070A7C83}" name="Project"/>
     <tableColumn id="2" xr3:uid="{E550573D-495D-FB4D-9952-E0A70DC9A0DD}" name="Country code"/>
     <tableColumn id="3" xr3:uid="{9607EDC7-8802-7840-AD53-E581C120BCE1}" name="Node code"/>
@@ -1083,6 +1096,7 @@
     <tableColumn id="7" xr3:uid="{33C9E816-ABF4-D94C-86A7-EC1574680166}" name="Coordinates"/>
     <tableColumn id="5" xr3:uid="{949981B5-0ABE-FD43-A1A8-8178B2562F0E}" name="size max (t)" dataDxfId="0" dataCellStyle="Comma"/>
     <tableColumn id="6" xr3:uid="{A3DDEF28-DE78-E047-A607-D6FCCE4682D6}" name="injection rate (t/hr)"/>
+    <tableColumn id="8" xr3:uid="{B5A3C7FA-B660-B043-858C-E82B43C2F92D}" name="Column1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2380,7 +2394,7 @@
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B57" t="s">
         <v>71</v>
@@ -2397,7 +2411,7 @@
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B58" t="s">
         <v>71</v>
@@ -2414,7 +2428,7 @@
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B59" t="s">
         <v>71</v>
@@ -3464,7 +3478,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDD3D8C9-E4BC-0046-BBBC-6939452B3EA0}">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13.83203125" customWidth="1"/>
@@ -3474,7 +3488,7 @@
     <col min="7" max="7" width="18.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="41" t="s">
         <v>197</v>
       </c>
@@ -3488,7 +3502,7 @@
         <v>200</v>
       </c>
       <c r="E1" s="41" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F1" s="41" t="s">
         <v>202</v>
@@ -3496,8 +3510,11 @@
       <c r="G1" s="41" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H1" s="41" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>62</v>
       </c>
@@ -3514,10 +3531,14 @@
         <v>240000000</v>
       </c>
       <c r="G2">
-        <v>2283</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+        <f>5000000/8760</f>
+        <v>570.77625570776252</v>
+      </c>
+      <c r="H2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>204</v>
       </c>
@@ -3533,11 +3554,12 @@
       <c r="F3" s="42">
         <v>550000000</v>
       </c>
-      <c r="G3">
-        <v>2968</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G3" s="44">
+        <f>9000000/8760</f>
+        <v>1027.3972602739725</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>93</v>
       </c>
@@ -3545,22 +3567,23 @@
         <v>72</v>
       </c>
       <c r="C4" t="s">
+        <v>209</v>
+      </c>
+      <c r="D4" t="s">
         <v>210</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>211</v>
-      </c>
-      <c r="E4" t="s">
-        <v>212</v>
       </c>
       <c r="F4" s="42">
         <v>125000000</v>
       </c>
-      <c r="G4">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G4" s="44">
+        <f>2500000/8760</f>
+        <v>285.38812785388126</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>205</v>
       </c>
@@ -3576,13 +3599,14 @@
       <c r="F5" s="42">
         <v>300000000</v>
       </c>
-      <c r="G5">
-        <v>1370</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G5" s="44">
+        <f>3600000/8760</f>
+        <v>410.95890410958901</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B6" t="s">
         <v>61</v>
@@ -3597,35 +3621,40 @@
         <v>1565000000</v>
       </c>
       <c r="G6">
-        <v>7991</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+        <f>(6000000+6000000+1500000)/8760</f>
+        <v>1541.0958904109589</v>
+      </c>
+      <c r="H6" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B7" t="s">
         <v>98</v>
       </c>
       <c r="C7" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D7" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F7" s="42">
         <v>720000000</v>
       </c>
-      <c r="G7">
-        <v>3425</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G7" s="44">
+        <f>(1500000+1500000+5000000)/8760</f>
+        <v>913.24200913242009</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B8" t="s">
         <v>61</v>
@@ -3640,10 +3669,11 @@
         <v>450000000</v>
       </c>
       <c r="G8">
-        <v>3539</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+        <f>(4000000+4000000)/8760</f>
+        <v>913.24200913242009</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>65</v>
       </c>
@@ -3660,12 +3690,13 @@
         <v>126000000</v>
       </c>
       <c r="G9">
-        <v>685</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+        <f>1000000/8760</f>
+        <v>114.15525114155251</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B10" t="s">
         <v>98</v>
@@ -3679,11 +3710,12 @@
       <c r="F10" s="42">
         <v>121000000</v>
       </c>
-      <c r="G10">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G10" s="44">
+        <f>4700000/8760</f>
+        <v>536.52968036529683</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>118</v>
       </c>
@@ -3699,34 +3731,36 @@
       <c r="F11" s="42">
         <v>37000000</v>
       </c>
-      <c r="G11">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G11" s="44">
+        <f>2500000/8760</f>
+        <v>285.38812785388126</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B12" t="s">
         <v>98</v>
       </c>
       <c r="C12" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D12" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E12" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F12" s="42">
         <v>225000000</v>
       </c>
-      <c r="G12">
-        <v>1027</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G12" s="44">
+        <f>3600000/8760</f>
+        <v>410.95890410958901</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>66</v>
       </c>
@@ -3743,12 +3777,13 @@
         <v>300000000</v>
       </c>
       <c r="G13">
-        <v>1712</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+        <f>4500000/8760</f>
+        <v>513.69863013698625</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>206</v>
+        <v>224</v>
       </c>
       <c r="B14" t="s">
         <v>98</v>
@@ -3760,13 +3795,14 @@
         <v>201</v>
       </c>
       <c r="F14" s="42">
-        <v>215000000</v>
-      </c>
-      <c r="G14">
-        <v>856</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+        <v>750000000</v>
+      </c>
+      <c r="G14" s="44">
+        <f>10000000/8760</f>
+        <v>1141.552511415525</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>68</v>
       </c>
@@ -3783,10 +3819,11 @@
         <v>500000000</v>
       </c>
       <c r="G15">
-        <v>913</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+        <f>900000/8760</f>
+        <v>102.73972602739725</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>95</v>
       </c>
@@ -3802,23 +3839,24 @@
       <c r="F16" s="42">
         <v>500000000</v>
       </c>
-      <c r="G16">
-        <v>913</v>
+      <c r="G16" s="44">
+        <f>1500000/8760</f>
+        <v>171.23287671232876</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" s="43" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="43" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>